<commit_message>
Pose de vrais hyperliens dans les courriels
Une adresse de deux cents caractères en plein paragraphe casse la mise en page
et se lit mal, surtout quand il y en a trois. Le proxy laissait passer le HTML
depuis le début, je ne m'en étais pas servi.

Les liens s'écrivent en markdown dans les constantes, ce qui garde le chiffrier
lisible, et `en_html` les convertit en balises juste avant de parler à Missive.
L'échappement des chevrons se fait avant la pose des balises, sinon on
échapperait ses propres liens.

Vérifié sur un brouillon déposé : Missive rend « notre média kit est ici
(https://…) » en texte, ce qui est exactement sa façon d'afficher une ancre,
la même que pour la signature de Gabriel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_brouillons_a_editer.xlsx
+++ b/communique-dragons/Lasclay_brouillons_a_editer.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>L'asclépiade à Dragons' Den le 17 septembre</t>
+          <t>L'asclépiade à Dragons' Den!</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2238,7 +2238,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vos lecteurs aimeraient voir comment une gousse devient un manteau.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2307,7 +2307,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2376,7 +2376,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2445,7 +2445,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2514,7 +2514,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2583,7 +2583,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2652,7 +2652,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2721,7 +2721,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2790,7 +2790,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2859,7 +2859,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2928,7 +2928,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2997,7 +2997,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3066,7 +3066,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3135,7 +3135,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3204,7 +3204,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3273,7 +3273,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3342,7 +3342,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3407,11 +3407,11 @@
           <t>Bonjour Catherine,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3479,7 +3479,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : huit ans après Saint-Tite, il reste quelque chose de cette promesse-là, et ça se raconte.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3548,7 +3548,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3617,7 +3617,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3686,7 +3686,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3755,7 +3755,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3824,7 +3824,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3893,7 +3893,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3962,7 +3962,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4031,7 +4031,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4100,7 +4100,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4169,7 +4169,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4238,7 +4238,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4307,7 +4307,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4376,7 +4376,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4445,7 +4445,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4514,7 +4514,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4583,7 +4583,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4648,11 +4648,11 @@
           <t>Bonjour Marianne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4721,7 +4721,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4790,7 +4790,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4859,7 +4859,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4928,7 +4928,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4997,7 +4997,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5066,7 +5066,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5135,7 +5135,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5204,7 +5204,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part parce que vos lecteurs ont vu la promesse de l'asclépiade de plus près que n'importe qui. Qui sait, peut-être vous inspirer un sujet sur ce que la plante est devenue depuis. Je peux parler des volumes, de la récolte, et de ce qui reste à régler.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5273,7 +5273,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5342,7 +5342,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5411,7 +5411,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5480,7 +5480,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5549,7 +5549,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5618,7 +5618,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5687,7 +5687,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5756,7 +5756,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5825,7 +5825,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5894,7 +5894,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5963,7 +5963,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6032,7 +6032,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6101,7 +6101,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6170,7 +6170,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6239,7 +6239,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6308,7 +6308,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6377,7 +6377,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6446,7 +6446,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6515,7 +6515,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6584,7 +6584,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6653,7 +6653,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6718,11 +6718,11 @@
           <t>Bonjour Scott,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6791,7 +6791,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6860,7 +6860,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6925,11 +6925,11 @@
           <t>Bonjour Karine,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6998,7 +6998,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7067,7 +7067,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7136,7 +7136,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7205,7 +7205,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7274,7 +7274,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7343,7 +7343,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7412,7 +7412,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7481,7 +7481,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7550,7 +7550,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7615,11 +7615,11 @@
           <t>Bonjour Pierre,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7688,7 +7688,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7757,7 +7757,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7826,7 +7826,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7895,7 +7895,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7964,7 +7964,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8033,7 +8033,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8102,7 +8102,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8171,7 +8171,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8240,7 +8240,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8309,7 +8309,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8378,7 +8378,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8447,7 +8447,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8516,7 +8516,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8585,7 +8585,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8654,7 +8654,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8723,7 +8723,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8792,7 +8792,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8861,7 +8861,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8926,12 +8926,12 @@
           <t>Bonjour Chloé,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, la MRC de Mékinac a fait pencher la relance (https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
+Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, [la MRC de Mékinac a fait pencher la relance](https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
 Neuf ans après, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Ce jeudi, c'est cette plante-là que je vais défendre à la télévision nationale.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9000,7 +9000,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9069,7 +9069,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9138,7 +9138,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9207,7 +9207,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9272,12 +9272,12 @@
           <t>Bonjour Jacinthe,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, la MRC de Mékinac a fait pencher la relance (https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
+Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, [la MRC de Mékinac a fait pencher la relance](https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
 Neuf ans après, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Ce jeudi, c'est cette plante-là que je vais défendre à la télévision nationale.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9346,7 +9346,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9411,11 +9411,11 @@
           <t>Bonjour Yvan,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9480,11 +9480,11 @@
           <t>Bonjour Yves,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9553,7 +9553,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9622,7 +9622,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9691,7 +9691,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9760,7 +9760,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9829,7 +9829,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9898,7 +9898,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9967,7 +9967,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10036,7 +10036,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10101,11 +10101,11 @@
           <t>Bonjour Carole,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après la faillite d'octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
+Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après [la faillite d'octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10174,7 +10174,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10243,7 +10243,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10312,7 +10312,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10381,7 +10381,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10450,7 +10450,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10519,7 +10519,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10584,11 +10584,11 @@
           <t>Bonjour Michel,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après la faillite d'octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
+Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après [la faillite d'octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10657,7 +10657,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10726,7 +10726,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10795,7 +10795,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10860,12 +10860,12 @@
           <t>Bonjour Anick,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, la MRC de Mékinac a fait pencher la relance (https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
+Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, [la MRC de Mékinac a fait pencher la relance](https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
 Neuf ans après, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Ce jeudi, c'est cette plante-là que je vais défendre à la télévision nationale.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10934,7 +10934,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11003,7 +11003,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11068,11 +11068,11 @@
           <t>Bonjour Julia,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après la faillite d'octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
+Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après [la faillite d'octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11141,7 +11141,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11210,7 +11210,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11279,7 +11279,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11348,7 +11348,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11417,7 +11417,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11486,7 +11486,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11555,7 +11555,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11624,7 +11624,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11693,7 +11693,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11762,7 +11762,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11831,7 +11831,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11900,7 +11900,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11969,7 +11969,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12038,7 +12038,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12107,7 +12107,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12176,7 +12176,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12245,7 +12245,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12314,7 +12314,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12383,7 +12383,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12452,7 +12452,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12521,7 +12521,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12590,7 +12590,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12655,11 +12655,11 @@
           <t>Bonjour Thomas,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12728,7 +12728,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12797,7 +12797,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12866,7 +12866,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12935,7 +12935,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13004,7 +13004,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13073,7 +13073,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13142,7 +13142,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13211,7 +13211,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13280,7 +13280,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13349,7 +13349,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13418,7 +13418,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13487,7 +13487,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13556,7 +13556,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13625,7 +13625,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13694,7 +13694,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13763,7 +13763,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13832,7 +13832,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13901,7 +13901,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13970,7 +13970,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14039,7 +14039,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14108,7 +14108,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14177,7 +14177,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14246,7 +14246,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14315,7 +14315,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14384,7 +14384,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14453,7 +14453,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14522,7 +14522,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14591,7 +14591,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14660,7 +14660,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14729,7 +14729,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14798,7 +14798,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14867,7 +14867,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14932,11 +14932,11 @@
           <t>Bonjour Timothy,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après la faillite d'octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
+Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après [la faillite d'octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15005,7 +15005,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15074,7 +15074,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15143,7 +15143,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15208,11 +15208,11 @@
           <t>Bonjour Isaac,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après la faillite d'octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
+Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après [la faillite d'octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15281,7 +15281,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15350,7 +15350,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15419,7 +15419,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15488,7 +15488,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15557,7 +15557,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15626,7 +15626,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15695,7 +15695,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15764,7 +15764,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15833,7 +15833,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15898,11 +15898,11 @@
           <t>Bonjour Louis-Philippe,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après la faillite d'octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
+Je vous écris parce que l'asclépiade se cultive chez vous depuis la première vague de 2013, celle de la Coopérative Monark et de ses 125 producteurs. Plusieurs de ceux qui ont tenu bon après [la faillite d'octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) nous vendent encore leur récolte.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15971,7 +15971,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16040,7 +16040,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16109,7 +16109,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16178,7 +16178,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16247,7 +16247,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16316,7 +16316,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16385,7 +16385,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16454,7 +16454,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16523,7 +16523,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16592,7 +16592,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16661,7 +16661,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16730,7 +16730,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16795,12 +16795,12 @@
           <t>Bonjour Paule,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, la MRC de Mékinac a fait pencher la relance (https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
+Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, [la MRC de Mékinac a fait pencher la relance](https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
 Neuf ans après, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Ce jeudi, c'est cette plante-là que je vais défendre à la télévision nationale.
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16869,7 +16869,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16938,7 +16938,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17007,7 +17007,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17076,7 +17076,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17145,7 +17145,7 @@
 Ce jeudi 17 septembre, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17212,7 +17212,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 I'm writing to the wire first because if this is worth two paragraphs, it's worth them in every paper in the country: a Quebec company insulating winter coats with the only plant monarch caterpillars can eat is going on national television Thursday.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17285,7 +17285,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 The business story: we built our own processing because no subcontractor would touch the fibre, changed our manufacturing model last year to survive, and are now pitching on national television.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17358,7 +17358,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Quebec company built its own processing because no subcontractor would touch the fibre, changed its manufacturing model last year to survive, and is now pitching on national television. Whatever happens in the episode, the fibre and the farms behind it are real.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17431,7 +17431,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars eat.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17504,7 +17504,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars eat.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17577,7 +17577,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 We're a Quebec City company, the milkweed is grown by Quebec farmers, and the insulation is made here, Thursday's national broadcast is a local story first.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17650,7 +17650,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 We're a Canadian direct-to-consumer brand about to get national television exposure, with a supply chain that starts in Quebec fields. The coat on the shelf begins as a pod in a row of weeds somebody decided not to spray.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17698,7 +17698,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>You covered Vegeto's milkweed insulation last February. We're the other end of that same Quebec filière: we buy the harvest, process the floss into insulation ourselves, and sell finished garments. As far as we know, nobody else holds the whole chain. The Quebec filière collapsed on October 11, 2017 when the group that had reserved 90 per cent of the crop went bankrupt (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), which is the context for anything written about milkweed insulation today.</t>
+          <t>You covered Vegeto's milkweed insulation last February. We're the other end of that same Quebec filière: we buy the harvest, process the floss into insulation ourselves, and sell finished garments. As far as we know, nobody else holds the whole chain. The Quebec filière collapsed [on October 11, 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) when the group that had reserved 90 per cent of the crop went bankrupt, which is the context for anything written about milkweed insulation today.</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -17721,9 +17721,9 @@
           <t>Hello,
 My name is Gabriel Gouveia, founder of Lasclay. We insulate winter clothing with a weed called milkweed, which we grow to help save an emblematic, threatened pollinator: the monarch butterfly.
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
-You covered Vegeto's milkweed insulation last February. We're the other end of that same Quebec filière: we buy the harvest, process the floss into insulation ourselves, and sell finished garments. As far as we know, nobody else holds the whole chain. The Quebec filière collapsed on October 11, 2017 when the group that had reserved 90 per cent of the crop went bankrupt (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), which is the context for anything written about milkweed insulation today.
+You covered Vegeto's milkweed insulation last February. We're the other end of that same Quebec filière: we buy the harvest, process the floss into insulation ourselves, and sell finished garments. As far as we know, nobody else holds the whole chain. The Quebec filière collapsed [on October 11, 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark) when the group that had reserved 90 per cent of the crop went bankrupt, which is the context for anything written about milkweed insulation today.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17796,7 +17796,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Milkweed floss is a hollow, naturally water-repellent fibre that behaves like down without an animal. A Quebec filière has been trying to industrialise it since 2013; we process it ourselves and sell finished garments.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17869,7 +17869,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Milkweed floss is a hollow, naturally water-repellent fibre that behaves like down without an animal, and a Quebec filière has been trying to industrialise it since 2013. We process it ourselves and sell finished garments. That last step is where the earlier attempts stopped.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -17942,7 +17942,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Plant-based insulation is one of the few places where outerwear can actually leave animal and petroleum fibres behind, and milkweed is the rare one that also feeds a threatened pollinator.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18015,7 +18015,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18088,7 +18088,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18161,7 +18161,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18234,7 +18234,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18307,7 +18307,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18380,7 +18380,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18453,7 +18453,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18526,7 +18526,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A Canadian company goes on Dragons' Den this Thursday with a winter coat insulated by a weed most farmers spray, and that same weed is the only thing monarch caterpillars can eat. We grow it, we process the floss into insulation ourselves in Quebec City, and we sell the finished garments across the country.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18599,7 +18599,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 A $300 winter coat insulated with a farm weed instead of down or polyester. The consumer question is whether it actually keeps you warm, and that is a fair thing to test on air.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18672,7 +18672,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers can watch it Thursday night. The milkweed is grown by Quebec farmers and the floss is processed into insulation in Quebec City. Final assembly of the garments happens offshore, which is what put the coat near $300 instead of the $1,000 the earlier attempts asked.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18745,7 +18745,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers can watch it Thursday night. The milkweed is grown by Quebec farmers and the floss is processed into insulation in Quebec City. Final assembly of the garments happens offshore, which is what put the coat near $300 instead of the $1,000 the earlier attempts asked.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18818,7 +18818,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers can watch it Thursday night. The milkweed is grown by Quebec farmers and the floss is processed into insulation in Quebec City. Final assembly of the garments happens offshore, which is what put the coat near $300 instead of the $1,000 the earlier attempts asked.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18891,7 +18891,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers can watch it Thursday night. The milkweed is grown by Quebec farmers and the floss is processed into insulation in Quebec City. Final assembly of the garments happens offshore, which is what put the coat near $300 instead of the $1,000 the earlier attempts asked.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -18964,7 +18964,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers can watch it Thursday night. The milkweed is grown by Quebec farmers and the floss is processed into insulation in Quebec City. Final assembly of the garments happens offshore, which is what put the coat near $300 instead of the $1,000 the earlier attempts asked.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19037,7 +19037,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Milkweed floss is a hollow, naturally water-repellent fibre that behaves like down without an animal. A Quebec filière has been trying to industrialise it since 2013; we process it ourselves and sell finished garments, which is the part nobody had managed to hold.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19110,7 +19110,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 The business angle from the Atlantic side: we built our own processing because no subcontractor would touch the fibre, and we are about to pitch it on national television. Atlantic Canada has the same problem we had, a raw material with no processing chain.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19183,7 +19183,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers buy winter coats to work in, not to walk to the car. Ours is insulated with a plant fibre instead of down or polyester, and I would rather have it judged by people who actually need it to hold at forty below than by anyone in a city. I'll send one to a reporter who wants to try it and say publicly what they found, good or bad.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19256,7 +19256,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers buy winter coats to work in, not to walk to the car. Ours is insulated with a plant fibre instead of down or polyester, and I would rather have it judged by people who actually need it to hold at forty below than by anyone in a city. I'll send one to a reporter who wants to try it and say publicly what they found, good or bad.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19329,7 +19329,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers buy winter coats to work in, not to walk to the car. Ours is insulated with a plant fibre instead of down or polyester, and I would rather have it judged by people who actually need it to hold at forty below than by anyone in a city. I'll send one to a reporter who wants to try it and say publicly what they found, good or bad.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19402,7 +19402,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 Your readers buy winter coats to work in, not to walk to the car. Ours is insulated with a plant fibre instead of down or polyester, and I would rather have it judged by people who actually need it to hold at forty below than by anyone in a city. I'll send one to a reporter who wants to try it and say publicly what they found, good or bad.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19475,7 +19475,7 @@
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
 The farm side of it: milkweed is a weed most growers spray, and a Quebec cooperative of 125 producers lost its only buyer overnight in 2017. We still buy the harvest. That question, whether anyone is waiting at the end of the field, is not specific to Quebec.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19523,7 +19523,7 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>The farm side: milkweed is a weed most growers spray, and a Quebec filière has been trying since 2013 to make it pay at the field gate. It stopped on October 11, 2017, when the group that had reserved 90 per cent of the Quebec crop went bankrupt and 125 growers lost their buyer overnight (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). We still buy the harvest, and that is the part that decides whether anyone plants it again.</t>
+          <t>The farm side: milkweed is a weed most growers spray, and a Quebec filière has been trying since 2013 to make it pay at the field gate. It stopped on October 11, 2017, when the group that had reserved 90 per cent of the Quebec crop went bankrupt and 125 growers lost their buyer overnight[, as Radio-Canada reported at the time](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). We still buy the harvest, and that is the part that decides whether anyone plants it again.</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
@@ -19546,9 +19546,9 @@
           <t>Hello,
 My name is Gabriel Gouveia, founder of Lasclay. We insulate winter clothing with a weed called milkweed, which we grow to help save an emblematic, threatened pollinator: the monarch butterfly.
 Its pods are filled with a hollow floss, very light and naturally water-repellent. We turn it into insulation in Quebec City and put it into coats, mitts, toques and cooler bags sold across Canada and the United States.
-The farm side: milkweed is a weed most growers spray, and a Quebec filière has been trying since 2013 to make it pay at the field gate. It stopped on October 11, 2017, when the group that had reserved 90 per cent of the Quebec crop went bankrupt and 125 growers lost their buyer overnight (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). We still buy the harvest, and that is the part that decides whether anyone plants it again.
+The farm side: milkweed is a weed most growers spray, and a Quebec filière has been trying since 2013 to make it pay at the field gate. It stopped on October 11, 2017, when the group that had reserved 90 per cent of the Quebec crop went bankrupt and 125 growers lost their buyer overnight[, as Radio-Canada reported at the time](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). We still buy the harvest, and that is the part that decides whether anyone plants it again.
 This Thursday, September 17, Lasclay is in the first episode of season 21 of Dragons' Den, on CBC and CBC Gem at 8 p.m. (8:30 NT).
-If you'd like to cover it, or a colleague might, our media kit is here, with images from the Dragons' Den floor and of the company: https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+If you'd like to cover it, or a colleague might, [our media kit is here](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), with images from the Dragons' Den floor and of the company.
 I'm hoping this visibility moves sales, which more broadly is very good news for the Quebec milkweed growers we keep buying from, and for the threatened monarchs that keep breeding in their fields.
 Happy to answer any questions, and available for an interview this week.
 Warmly,
@@ -19614,11 +19614,11 @@
           <t>Bonjour Johanne,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -19684,11 +19684,11 @@
           <t>Bonjour Catherine,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -19754,11 +19754,11 @@
           <t>Bonjour France,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -19824,11 +19824,11 @@
           <t>Bonjour Gilbert,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -19894,11 +19894,11 @@
           <t>Bonjour Carine,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -19964,11 +19964,11 @@
           <t>Bonjour Maxime,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20034,11 +20034,11 @@
           <t>Bonjour Marie,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20104,11 +20104,11 @@
           <t>Bonjour Julie,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20174,11 +20174,11 @@
           <t>Bonjour Marc-Yvan,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20244,11 +20244,11 @@
           <t>Bonjour Benoit,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
+Je vous écris parce que l'asclépiade est une histoire agricole avec une date de rupture. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3 et avait réservé 90 % de la récolte québécoise, a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark). Les 125 producteurs de la Coopérative Monark se sont retrouvés sans acheteur, et la question n'a pas changé depuis : y a-t-il quelqu'un au bout du champ.
 Nous, on achète encore. Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive pour nous depuis nos tout débuts, et je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20317,7 +20317,7 @@
 Je vous écris parce que c'est d'abord une histoire d'affaires : bâtir ses propres procédés faute de sous-traitant prêt à toucher à la fibre, puis changer de modèle manufacturier l'an dernier pour tenir, et se retrouver à pitcher à la télévision nationale. La vidéo sur le changement de modèle est ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20386,7 +20386,7 @@
 Notre atelier est à Québec, et c'est là que la soie d'asclépiade devient de l'isolant.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20455,7 +20455,7 @@
 Je vous écris parce que Sabin Tremblay, à L'Ascension-de-Notre-Seigneur, cultive de l'asclépiade pour nous depuis nos tout débuts, et qu'il en cultive encore. Je vais l'aider à récolter le 4 octobre. S'il y a un reportage à faire, il est là autant qu'ici.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20521,11 +20521,11 @@
           <t>Bonjour,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite le 11 octobre 2017 (https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, la MRC de Mékinac a fait pencher la relance (https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
+Je vous écris parce que l'asclépiade a commencé chez vous, à Saint-Tite et dans Mékinac. Le groupe Protec-Style, qui exploitait l'usine de Saint-Tite sous le nom d'Encore 3, avait réservé 90 % de la récolte québécoise quand il a fait faillite [le 11 octobre 2017](https://ici.radio-canada.ca/nouvelle/1061543/asclepiade-soyer-producteurs-industries-encore3-faillite-monark), emportant Saint-Tite et son atelier de Granby. Les 125 producteurs de la Coopérative Monark ont pris le choc. Six semaines plus tard, [la MRC de Mékinac a fait pencher la relance](https://lenouvelliste.ca/affaires/asclepiade-les-activites-reprennent-a-lusine-de-saint-tite-9a7c0d08d77c81c7ab22fdfc8e47a922).
 Neuf ans après, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Ce jeudi, c'est cette plante-là que je vais défendre à la télévision nationale.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20591,10 +20591,10 @@
           <t>Bonjour,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
 Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
-Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées le 11 octobre 2017 avec une dette de plus de 1,4 M$ (https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/). L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
+Je vous écris parce que la transformation de la fibre se faisait à Granby, rue Bernard. L'atelier appartenait au groupe Protec-Style, qui exploitait aussi l'usine de Saint-Tite, et les deux sont tombées [le 11 octobre 2017](https://www.lhebdodustmaurice.com/actualite/protec-style-en-faillite/) avec une dette de plus de 1,4 M$. L'Estrie compte encore des producteurs d'asclépiade, et on continue d'acheter de la fibre québécoise.
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20663,7 +20663,7 @@
 Je vous écris parce que c'est d'abord une histoire d'affaires : bâtir ses propres procédés faute de sous-traitant prêt à toucher à la fibre, puis changer de modèle manufacturier l'an dernier pour tenir, et se retrouver à pitcher à la télévision nationale. La vidéo sur le changement de modèle est ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20732,7 +20732,7 @@
 Je vous écris parce que c'est d'abord une histoire d'affaires : bâtir ses propres procédés faute de sous-traitant prêt à toucher à la fibre, puis changer de modèle manufacturier l'an dernier pour tenir, et se retrouver à pitcher à la télévision nationale. La vidéo sur le changement de modèle est ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20801,7 +20801,7 @@
 Je vous écris parce que c'est d'abord une histoire d'affaires : bâtir ses propres procédés faute de sous-traitant prêt à toucher à la fibre, puis changer de modèle manufacturier l'an dernier pour tenir, et se retrouver à pitcher à la télévision nationale. La vidéo sur le changement de modèle est ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20870,7 +20870,7 @@
 Je vous écris parce que c'est d'abord une histoire d'affaires : bâtir ses propres procédés faute de sous-traitant prêt à toucher à la fibre, puis changer de modèle manufacturier l'an dernier pour tenir, et se retrouver à pitcher à la télévision nationale. La vidéo sur le changement de modèle est ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -20939,7 +20939,7 @@
 Je vous écris parce que c'est d'abord une histoire d'affaires : bâtir ses propres procédés faute de sous-traitant prêt à toucher à la fibre, puis changer de modèle manufacturier l'an dernier pour tenir, et se retrouver à pitcher à la télévision nationale. La vidéo sur le changement de modèle est ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,
@@ -21008,7 +21008,7 @@
 Je vous écris parce que c'est d'abord une histoire d'affaires : bâtir ses propres procédés faute de sous-traitant prêt à toucher à la fibre, puis changer de modèle manufacturier l'an dernier pour tenir, et se retrouver à pitcher à la télévision nationale. La vidéo sur le changement de modèle est ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU
 Ce jeudi 17 septembre, je présente Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem, à 20 h.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue d'ici jeudi, ou le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+Si ça vous intéresse de couvrir (ou un.e collègue?), [notre média kit est ici](https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr), avec les images de notre passage à Dragons' Den et de l'entreprise.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.
 Chaleureusement,

</xml_diff>